<commit_message>
Add support for optional login ID alongside email for user authentication
- Updated login functionality to accept either login ID or email.
- Modified user model to include optional login ID field.
- Adjusted admin user management to handle login IDs.
- Enhanced seeding script to backfill login IDs for existing users.
- Updated README with new login instructions.
</commit_message>
<xml_diff>
--- a/sample-data/pos-minmax-bar.xlsx
+++ b/sample-data/pos-minmax-bar.xlsx
@@ -430,13 +430,13 @@
         <v>btl</v>
       </c>
       <c r="D2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -450,13 +450,13 @@
         <v>btl</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -470,13 +470,13 @@
         <v>btl</v>
       </c>
       <c r="D4">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E4">
         <v>2</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -490,13 +490,13 @@
         <v>btl</v>
       </c>
       <c r="D5">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -510,13 +510,13 @@
         <v>btl</v>
       </c>
       <c r="D6">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -530,13 +530,13 @@
         <v>btl</v>
       </c>
       <c r="D7">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -570,13 +570,13 @@
         <v>btl</v>
       </c>
       <c r="D9">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -590,13 +590,13 @@
         <v>btl</v>
       </c>
       <c r="D10">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -610,13 +610,13 @@
         <v>btl</v>
       </c>
       <c r="D11">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate sample POS files from seed run
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-data/pos-minmax-bar.xlsx
+++ b/sample-data/pos-minmax-bar.xlsx
@@ -430,13 +430,13 @@
         <v>btl</v>
       </c>
       <c r="D2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -450,13 +450,13 @@
         <v>btl</v>
       </c>
       <c r="D3">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -470,13 +470,13 @@
         <v>btl</v>
       </c>
       <c r="D4">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E4">
         <v>2</v>
       </c>
       <c r="F4">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -490,13 +490,13 @@
         <v>btl</v>
       </c>
       <c r="D5">
+        <v>17</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5">
         <v>7</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -510,13 +510,13 @@
         <v>btl</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -533,10 +533,10 @@
         <v>11</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -550,13 +550,13 @@
         <v>btl</v>
       </c>
       <c r="D8">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -570,10 +570,10 @@
         <v>btl</v>
       </c>
       <c r="D9">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -593,10 +593,10 @@
         <v>16</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -610,13 +610,13 @@
         <v>btl</v>
       </c>
       <c r="D11">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>